<commit_message>
refactoring enemies  animations structure and adding new eney
</commit_message>
<xml_diff>
--- a/initial_enemies_stats.xlsx
+++ b/initial_enemies_stats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\godot\rpg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A102E449-76AA-4583-AEEF-AB2C00D988A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9760BBE3-F3F5-4611-93C9-BD35C27D02D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -404,11 +404,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -726,7 +726,7 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="6" t="s">
         <v>25</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -755,7 +755,7 @@
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="7"/>
+      <c r="A3" s="6"/>
       <c r="B3" s="3"/>
       <c r="C3" s="5"/>
       <c r="D3" s="5"/>
@@ -766,7 +766,7 @@
       <c r="I3" s="5"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="7"/>
+      <c r="A4" s="6"/>
       <c r="B4" s="2" t="s">
         <v>26</v>
       </c>
@@ -779,917 +779,1020 @@
       <c r="I4" s="5"/>
     </row>
     <row r="5" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="6" t="s">
         <v>25</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="7">
         <v>160</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="7">
         <v>32</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="7">
         <v>45</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="7">
         <v>14</v>
       </c>
-      <c r="G5" s="6">
+      <c r="G5" s="7">
         <v>1.5</v>
       </c>
-      <c r="H5" s="6">
+      <c r="H5" s="7">
         <v>1</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="I5" s="7" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="7"/>
+      <c r="A6" s="6"/>
       <c r="B6" s="3"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="7"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="7"/>
+      <c r="A7" s="6"/>
       <c r="B7" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
     </row>
     <row r="8" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="6" t="s">
         <v>25</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="7">
         <v>110</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="7">
         <v>35</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="7">
         <v>75</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="7">
         <v>11</v>
       </c>
-      <c r="G8" s="6">
+      <c r="G8" s="7">
         <v>1.1000000000000001</v>
       </c>
-      <c r="H8" s="6">
+      <c r="H8" s="7">
         <v>0.75</v>
       </c>
-      <c r="I8" s="6" t="s">
+      <c r="I8" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="7"/>
+      <c r="A9" s="6"/>
       <c r="B9" s="3"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="7"/>
+      <c r="A10" s="6"/>
       <c r="B10" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
     </row>
     <row r="11" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="6" t="s">
         <v>25</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="7">
         <v>80</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="7">
         <v>24</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="7">
         <v>40</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="7">
         <v>8</v>
       </c>
-      <c r="G11" s="6">
+      <c r="G11" s="7">
         <v>1.8</v>
       </c>
-      <c r="H11" s="6">
+      <c r="H11" s="7">
         <v>0.6</v>
       </c>
-      <c r="I11" s="6" t="s">
+      <c r="I11" s="7" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="7"/>
+      <c r="A12" s="6"/>
       <c r="B12" s="3"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="7"/>
+      <c r="A13" s="6"/>
       <c r="B13" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
     </row>
     <row r="14" spans="1:9" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="6" t="s">
         <v>25</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C14" s="6">
+      <c r="C14" s="7">
         <v>75</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="7">
         <v>50</v>
       </c>
-      <c r="F14" s="6">
+      <c r="F14" s="7">
         <v>12</v>
       </c>
-      <c r="G14" s="6">
+      <c r="G14" s="7">
         <v>1.4</v>
       </c>
-      <c r="H14" s="6">
+      <c r="H14" s="7">
         <v>0.9</v>
       </c>
-      <c r="I14" s="6" t="s">
+      <c r="I14" s="7" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" s="7"/>
+      <c r="A15" s="6"/>
       <c r="B15" s="3"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="6"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" s="7"/>
+      <c r="A16" s="6"/>
       <c r="B16" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
-      <c r="I16" s="6"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="7"/>
     </row>
     <row r="17" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="6" t="s">
         <v>25</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C17" s="6">
+      <c r="C17" s="7">
         <v>90</v>
       </c>
-      <c r="D17" s="6">
+      <c r="D17" s="7">
         <v>45</v>
       </c>
-      <c r="E17" s="6">
+      <c r="E17" s="7">
         <v>70</v>
       </c>
-      <c r="F17" s="6">
+      <c r="F17" s="7">
         <v>9</v>
       </c>
-      <c r="G17" s="6">
+      <c r="G17" s="7">
         <v>1</v>
       </c>
-      <c r="H17" s="6">
+      <c r="H17" s="7">
         <v>0.7</v>
       </c>
-      <c r="I17" s="6" t="s">
+      <c r="I17" s="7" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A18" s="7"/>
+      <c r="A18" s="6"/>
       <c r="B18" s="3"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="6"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="7"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" s="7"/>
+      <c r="A19" s="6"/>
       <c r="B19" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
-      <c r="I19" s="6"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="7"/>
     </row>
     <row r="20" spans="1:9" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="6" t="s">
         <v>25</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C20" s="6">
+      <c r="C20" s="7">
         <v>85</v>
       </c>
-      <c r="D20" s="6">
+      <c r="D20" s="7">
         <v>30</v>
       </c>
-      <c r="E20" s="6">
+      <c r="E20" s="7">
         <v>80</v>
       </c>
-      <c r="F20" s="6">
+      <c r="F20" s="7">
         <v>11.5</v>
       </c>
-      <c r="G20" s="6">
+      <c r="G20" s="7">
         <v>0.9</v>
       </c>
-      <c r="H20" s="6">
+      <c r="H20" s="7">
         <v>0.65</v>
       </c>
-      <c r="I20" s="6" t="s">
+      <c r="I20" s="7" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A21" s="7"/>
+      <c r="A21" s="6"/>
       <c r="B21" s="3"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
-      <c r="I21" s="6"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="7"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="7"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A22" s="7"/>
+      <c r="A22" s="6"/>
       <c r="B22" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="6"/>
-      <c r="I22" s="6"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="7"/>
     </row>
     <row r="23" spans="1:9" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A23" s="7" t="s">
+      <c r="A23" s="6" t="s">
         <v>35</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C23" s="6">
+      <c r="C23" s="7">
         <v>450</v>
       </c>
-      <c r="D23" s="6">
+      <c r="D23" s="7">
         <v>48</v>
       </c>
-      <c r="E23" s="6">
+      <c r="E23" s="7">
         <v>40</v>
       </c>
-      <c r="F23" s="6">
+      <c r="F23" s="7">
         <v>25</v>
       </c>
-      <c r="G23" s="6">
+      <c r="G23" s="7">
         <v>2</v>
       </c>
-      <c r="H23" s="6">
+      <c r="H23" s="7">
         <v>1.2</v>
       </c>
-      <c r="I23" s="6" t="s">
+      <c r="I23" s="7" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A24" s="7"/>
+      <c r="A24" s="6"/>
       <c r="B24" s="3"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
-      <c r="H24" s="6"/>
-      <c r="I24" s="6"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="7"/>
+      <c r="G24" s="7"/>
+      <c r="H24" s="7"/>
+      <c r="I24" s="7"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" s="7"/>
+      <c r="A25" s="6"/>
       <c r="B25" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
-      <c r="H25" s="6"/>
-      <c r="I25" s="6"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
+      <c r="H25" s="7"/>
+      <c r="I25" s="7"/>
     </row>
     <row r="26" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="7" t="s">
+      <c r="A26" s="6" t="s">
         <v>35</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="6">
+      <c r="C26" s="7">
         <v>65</v>
       </c>
-      <c r="D26" s="6">
+      <c r="D26" s="7">
         <v>22</v>
       </c>
-      <c r="E26" s="6">
+      <c r="E26" s="7">
         <v>90</v>
       </c>
-      <c r="F26" s="6">
+      <c r="F26" s="7">
         <v>7.5</v>
       </c>
-      <c r="G26" s="6">
+      <c r="G26" s="7">
         <v>0.7</v>
       </c>
-      <c r="H26" s="6">
+      <c r="H26" s="7">
         <v>0.5</v>
       </c>
-      <c r="I26" s="6" t="s">
+      <c r="I26" s="7" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" s="7"/>
+      <c r="A27" s="6"/>
       <c r="B27" s="3"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
-      <c r="E27" s="6"/>
-      <c r="F27" s="6"/>
-      <c r="G27" s="6"/>
-      <c r="H27" s="6"/>
-      <c r="I27" s="6"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="7"/>
+      <c r="E27" s="7"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="7"/>
+      <c r="H27" s="7"/>
+      <c r="I27" s="7"/>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A28" s="7"/>
+      <c r="A28" s="6"/>
       <c r="B28" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C28" s="6"/>
-      <c r="D28" s="6"/>
-      <c r="E28" s="6"/>
-      <c r="F28" s="6"/>
-      <c r="G28" s="6"/>
-      <c r="H28" s="6"/>
-      <c r="I28" s="6"/>
+      <c r="C28" s="7"/>
+      <c r="D28" s="7"/>
+      <c r="E28" s="7"/>
+      <c r="F28" s="7"/>
+      <c r="G28" s="7"/>
+      <c r="H28" s="7"/>
+      <c r="I28" s="7"/>
     </row>
     <row r="29" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A29" s="7" t="s">
+      <c r="A29" s="6" t="s">
         <v>35</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C29" s="6">
+      <c r="C29" s="7">
         <v>95</v>
       </c>
-      <c r="D29" s="6">
+      <c r="D29" s="7">
         <v>30</v>
       </c>
-      <c r="E29" s="6">
+      <c r="E29" s="7">
         <v>70</v>
       </c>
-      <c r="F29" s="6" t="s">
+      <c r="F29" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="G29" s="6">
+      <c r="G29" s="7">
         <v>1.1000000000000001</v>
       </c>
-      <c r="H29" s="6">
+      <c r="H29" s="7">
         <v>0.7</v>
       </c>
-      <c r="I29" s="6" t="s">
+      <c r="I29" s="7" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A30" s="7"/>
+      <c r="A30" s="6"/>
       <c r="B30" s="3"/>
-      <c r="C30" s="6"/>
-      <c r="D30" s="6"/>
-      <c r="E30" s="6"/>
-      <c r="F30" s="6"/>
-      <c r="G30" s="6"/>
-      <c r="H30" s="6"/>
-      <c r="I30" s="6"/>
+      <c r="C30" s="7"/>
+      <c r="D30" s="7"/>
+      <c r="E30" s="7"/>
+      <c r="F30" s="7"/>
+      <c r="G30" s="7"/>
+      <c r="H30" s="7"/>
+      <c r="I30" s="7"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A31" s="7"/>
+      <c r="A31" s="6"/>
       <c r="B31" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
-      <c r="E31" s="6"/>
-      <c r="F31" s="6"/>
-      <c r="G31" s="6"/>
-      <c r="H31" s="6"/>
-      <c r="I31" s="6"/>
+      <c r="C31" s="7"/>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
+      <c r="F31" s="7"/>
+      <c r="G31" s="7"/>
+      <c r="H31" s="7"/>
+      <c r="I31" s="7"/>
     </row>
     <row r="32" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="7" t="s">
+      <c r="A32" s="6" t="s">
         <v>35</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C32" s="6">
+      <c r="C32" s="7">
         <v>130</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D32" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="E32" s="6">
+      <c r="E32" s="7">
         <v>55</v>
       </c>
-      <c r="F32" s="6">
+      <c r="F32" s="7">
         <v>13</v>
       </c>
-      <c r="G32" s="6">
+      <c r="G32" s="7">
         <v>1.3</v>
       </c>
-      <c r="H32" s="6">
+      <c r="H32" s="7">
         <v>0.85</v>
       </c>
-      <c r="I32" s="6" t="s">
+      <c r="I32" s="7" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A33" s="7"/>
+      <c r="A33" s="6"/>
       <c r="B33" s="3"/>
-      <c r="C33" s="6"/>
-      <c r="D33" s="6"/>
-      <c r="E33" s="6"/>
-      <c r="F33" s="6"/>
-      <c r="G33" s="6"/>
-      <c r="H33" s="6"/>
-      <c r="I33" s="6"/>
+      <c r="C33" s="7"/>
+      <c r="D33" s="7"/>
+      <c r="E33" s="7"/>
+      <c r="F33" s="7"/>
+      <c r="G33" s="7"/>
+      <c r="H33" s="7"/>
+      <c r="I33" s="7"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A34" s="7"/>
+      <c r="A34" s="6"/>
       <c r="B34" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C34" s="6"/>
-      <c r="D34" s="6"/>
-      <c r="E34" s="6"/>
-      <c r="F34" s="6"/>
-      <c r="G34" s="6"/>
-      <c r="H34" s="6"/>
-      <c r="I34" s="6"/>
+      <c r="C34" s="7"/>
+      <c r="D34" s="7"/>
+      <c r="E34" s="7"/>
+      <c r="F34" s="7"/>
+      <c r="G34" s="7"/>
+      <c r="H34" s="7"/>
+      <c r="I34" s="7"/>
     </row>
     <row r="35" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A35" s="7" t="s">
+      <c r="A35" s="6" t="s">
         <v>35</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C35" s="6">
+      <c r="C35" s="7">
         <v>60</v>
       </c>
-      <c r="D35" s="6" t="s">
+      <c r="D35" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="E35" s="6">
+      <c r="E35" s="7">
         <v>85</v>
       </c>
-      <c r="F35" s="6">
+      <c r="F35" s="7">
         <v>6.5</v>
       </c>
-      <c r="G35" s="6">
+      <c r="G35" s="7">
         <v>0.8</v>
       </c>
-      <c r="H35" s="6">
+      <c r="H35" s="7">
         <v>0.55000000000000004</v>
       </c>
-      <c r="I35" s="6" t="s">
+      <c r="I35" s="7" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A36" s="7"/>
+      <c r="A36" s="6"/>
       <c r="B36" s="3"/>
-      <c r="C36" s="6"/>
-      <c r="D36" s="6"/>
-      <c r="E36" s="6"/>
-      <c r="F36" s="6"/>
-      <c r="G36" s="6"/>
-      <c r="H36" s="6"/>
-      <c r="I36" s="6"/>
+      <c r="C36" s="7"/>
+      <c r="D36" s="7"/>
+      <c r="E36" s="7"/>
+      <c r="F36" s="7"/>
+      <c r="G36" s="7"/>
+      <c r="H36" s="7"/>
+      <c r="I36" s="7"/>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A37" s="7"/>
+      <c r="A37" s="6"/>
       <c r="B37" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C37" s="6"/>
-      <c r="D37" s="6"/>
-      <c r="E37" s="6"/>
-      <c r="F37" s="6"/>
-      <c r="G37" s="6"/>
-      <c r="H37" s="6"/>
-      <c r="I37" s="6"/>
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="7"/>
+      <c r="G37" s="7"/>
+      <c r="H37" s="7"/>
+      <c r="I37" s="7"/>
     </row>
     <row r="38" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A38" s="7" t="s">
+      <c r="A38" s="6" t="s">
         <v>35</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C38" s="6">
+      <c r="C38" s="7">
         <v>140</v>
       </c>
-      <c r="D38" s="6">
+      <c r="D38" s="7">
         <v>30</v>
       </c>
-      <c r="E38" s="6">
+      <c r="E38" s="7">
         <v>60</v>
       </c>
-      <c r="F38" s="6" t="s">
+      <c r="F38" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="G38" s="6">
+      <c r="G38" s="7">
         <v>0.9</v>
       </c>
-      <c r="H38" s="6">
+      <c r="H38" s="7">
         <v>0.8</v>
       </c>
-      <c r="I38" s="6" t="s">
+      <c r="I38" s="7" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A39" s="7"/>
+      <c r="A39" s="6"/>
       <c r="B39" s="3"/>
-      <c r="C39" s="6"/>
-      <c r="D39" s="6"/>
-      <c r="E39" s="6"/>
-      <c r="F39" s="6"/>
-      <c r="G39" s="6"/>
-      <c r="H39" s="6"/>
-      <c r="I39" s="6"/>
+      <c r="C39" s="7"/>
+      <c r="D39" s="7"/>
+      <c r="E39" s="7"/>
+      <c r="F39" s="7"/>
+      <c r="G39" s="7"/>
+      <c r="H39" s="7"/>
+      <c r="I39" s="7"/>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A40" s="7"/>
+      <c r="A40" s="6"/>
       <c r="B40" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C40" s="6"/>
-      <c r="D40" s="6"/>
-      <c r="E40" s="6"/>
-      <c r="F40" s="6"/>
-      <c r="G40" s="6"/>
-      <c r="H40" s="6"/>
-      <c r="I40" s="6"/>
+      <c r="C40" s="7"/>
+      <c r="D40" s="7"/>
+      <c r="E40" s="7"/>
+      <c r="F40" s="7"/>
+      <c r="G40" s="7"/>
+      <c r="H40" s="7"/>
+      <c r="I40" s="7"/>
     </row>
     <row r="41" spans="1:9" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A41" s="7" t="s">
+      <c r="A41" s="6" t="s">
         <v>35</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C41" s="6">
+      <c r="C41" s="7">
         <v>220</v>
       </c>
-      <c r="D41" s="6">
+      <c r="D41" s="7">
         <v>26</v>
       </c>
-      <c r="E41" s="6">
+      <c r="E41" s="7">
         <v>30</v>
       </c>
-      <c r="F41" s="6">
+      <c r="F41" s="7">
         <v>16</v>
       </c>
-      <c r="G41" s="6">
+      <c r="G41" s="7">
         <v>2.2000000000000002</v>
       </c>
-      <c r="H41" s="6">
+      <c r="H41" s="7">
         <v>1.1000000000000001</v>
       </c>
-      <c r="I41" s="6" t="s">
+      <c r="I41" s="7" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A42" s="7"/>
+      <c r="A42" s="6"/>
       <c r="B42" s="3"/>
-      <c r="C42" s="6"/>
-      <c r="D42" s="6"/>
-      <c r="E42" s="6"/>
-      <c r="F42" s="6"/>
-      <c r="G42" s="6"/>
-      <c r="H42" s="6"/>
-      <c r="I42" s="6"/>
+      <c r="C42" s="7"/>
+      <c r="D42" s="7"/>
+      <c r="E42" s="7"/>
+      <c r="F42" s="7"/>
+      <c r="G42" s="7"/>
+      <c r="H42" s="7"/>
+      <c r="I42" s="7"/>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A43" s="7"/>
+      <c r="A43" s="6"/>
       <c r="B43" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C43" s="6"/>
-      <c r="D43" s="6"/>
-      <c r="E43" s="6"/>
-      <c r="F43" s="6"/>
-      <c r="G43" s="6"/>
-      <c r="H43" s="6"/>
-      <c r="I43" s="6"/>
+      <c r="C43" s="7"/>
+      <c r="D43" s="7"/>
+      <c r="E43" s="7"/>
+      <c r="F43" s="7"/>
+      <c r="G43" s="7"/>
+      <c r="H43" s="7"/>
+      <c r="I43" s="7"/>
     </row>
     <row r="44" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A44" s="7" t="s">
+      <c r="A44" s="6" t="s">
         <v>45</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C44" s="6">
+      <c r="C44" s="7">
         <v>180</v>
       </c>
-      <c r="D44" s="6">
+      <c r="D44" s="7">
         <v>36</v>
       </c>
-      <c r="E44" s="6">
+      <c r="E44" s="7">
         <v>50</v>
       </c>
-      <c r="F44" s="6">
+      <c r="F44" s="7">
         <v>18</v>
       </c>
-      <c r="G44" s="6">
+      <c r="G44" s="7">
         <v>1.6</v>
       </c>
-      <c r="H44" s="6">
+      <c r="H44" s="7">
         <v>1</v>
       </c>
-      <c r="I44" s="6" t="s">
+      <c r="I44" s="7" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A45" s="7"/>
+      <c r="A45" s="6"/>
       <c r="B45" s="3"/>
-      <c r="C45" s="6"/>
-      <c r="D45" s="6"/>
-      <c r="E45" s="6"/>
-      <c r="F45" s="6"/>
-      <c r="G45" s="6"/>
-      <c r="H45" s="6"/>
-      <c r="I45" s="6"/>
+      <c r="C45" s="7"/>
+      <c r="D45" s="7"/>
+      <c r="E45" s="7"/>
+      <c r="F45" s="7"/>
+      <c r="G45" s="7"/>
+      <c r="H45" s="7"/>
+      <c r="I45" s="7"/>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A46" s="7"/>
+      <c r="A46" s="6"/>
       <c r="B46" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C46" s="6"/>
-      <c r="D46" s="6"/>
-      <c r="E46" s="6"/>
-      <c r="F46" s="6"/>
-      <c r="G46" s="6"/>
-      <c r="H46" s="6"/>
-      <c r="I46" s="6"/>
+      <c r="C46" s="7"/>
+      <c r="D46" s="7"/>
+      <c r="E46" s="7"/>
+      <c r="F46" s="7"/>
+      <c r="G46" s="7"/>
+      <c r="H46" s="7"/>
+      <c r="I46" s="7"/>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A47" s="7" t="s">
+      <c r="A47" s="6" t="s">
         <v>45</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C47" s="6">
+      <c r="C47" s="7">
         <v>70</v>
       </c>
-      <c r="D47" s="6">
+      <c r="D47" s="7">
         <v>28</v>
       </c>
-      <c r="E47" s="6">
+      <c r="E47" s="7">
         <v>80</v>
       </c>
-      <c r="F47" s="6">
+      <c r="F47" s="7">
         <v>8.5</v>
       </c>
-      <c r="G47" s="6">
+      <c r="G47" s="7">
         <v>0.8</v>
       </c>
-      <c r="H47" s="6">
+      <c r="H47" s="7">
         <v>0.6</v>
       </c>
-      <c r="I47" s="6" t="s">
+      <c r="I47" s="7" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A48" s="7"/>
+      <c r="A48" s="6"/>
       <c r="B48" s="3"/>
-      <c r="C48" s="6"/>
-      <c r="D48" s="6"/>
-      <c r="E48" s="6"/>
-      <c r="F48" s="6"/>
-      <c r="G48" s="6"/>
-      <c r="H48" s="6"/>
-      <c r="I48" s="6"/>
+      <c r="C48" s="7"/>
+      <c r="D48" s="7"/>
+      <c r="E48" s="7"/>
+      <c r="F48" s="7"/>
+      <c r="G48" s="7"/>
+      <c r="H48" s="7"/>
+      <c r="I48" s="7"/>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A49" s="7"/>
+      <c r="A49" s="6"/>
       <c r="B49" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C49" s="6"/>
-      <c r="D49" s="6"/>
-      <c r="E49" s="6"/>
-      <c r="F49" s="6"/>
-      <c r="G49" s="6"/>
-      <c r="H49" s="6"/>
-      <c r="I49" s="6"/>
+      <c r="C49" s="7"/>
+      <c r="D49" s="7"/>
+      <c r="E49" s="7"/>
+      <c r="F49" s="7"/>
+      <c r="G49" s="7"/>
+      <c r="H49" s="7"/>
+      <c r="I49" s="7"/>
     </row>
     <row r="50" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A50" s="7" t="s">
+      <c r="A50" s="6" t="s">
         <v>45</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C50" s="6">
+      <c r="C50" s="7">
         <v>85</v>
       </c>
-      <c r="D50" s="6">
+      <c r="D50" s="7">
         <v>22</v>
       </c>
-      <c r="E50" s="6">
+      <c r="E50" s="7">
         <v>95</v>
       </c>
-      <c r="F50" s="6">
+      <c r="F50" s="7">
         <v>13.5</v>
       </c>
-      <c r="G50" s="6">
+      <c r="G50" s="7">
         <v>0.75</v>
       </c>
-      <c r="H50" s="6">
+      <c r="H50" s="7">
         <v>0.5</v>
       </c>
-      <c r="I50" s="6" t="s">
+      <c r="I50" s="7" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A51" s="7"/>
+      <c r="A51" s="6"/>
       <c r="B51" s="3"/>
-      <c r="C51" s="6"/>
-      <c r="D51" s="6"/>
-      <c r="E51" s="6"/>
-      <c r="F51" s="6"/>
-      <c r="G51" s="6"/>
-      <c r="H51" s="6"/>
-      <c r="I51" s="6"/>
+      <c r="C51" s="7"/>
+      <c r="D51" s="7"/>
+      <c r="E51" s="7"/>
+      <c r="F51" s="7"/>
+      <c r="G51" s="7"/>
+      <c r="H51" s="7"/>
+      <c r="I51" s="7"/>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A52" s="7"/>
+      <c r="A52" s="6"/>
       <c r="B52" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C52" s="6"/>
-      <c r="D52" s="6"/>
-      <c r="E52" s="6"/>
-      <c r="F52" s="6"/>
-      <c r="G52" s="6"/>
-      <c r="H52" s="6"/>
-      <c r="I52" s="6"/>
+      <c r="C52" s="7"/>
+      <c r="D52" s="7"/>
+      <c r="E52" s="7"/>
+      <c r="F52" s="7"/>
+      <c r="G52" s="7"/>
+      <c r="H52" s="7"/>
+      <c r="I52" s="7"/>
     </row>
     <row r="53" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A53" s="7" t="s">
+      <c r="A53" s="6" t="s">
         <v>49</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C53" s="6">
+      <c r="C53" s="7">
         <v>800</v>
       </c>
-      <c r="D53" s="6">
+      <c r="D53" s="7">
         <v>55</v>
       </c>
-      <c r="E53" s="6">
+      <c r="E53" s="7">
         <v>35</v>
       </c>
-      <c r="F53" s="6" t="s">
+      <c r="F53" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="G53" s="6">
+      <c r="G53" s="7">
         <v>2.5</v>
       </c>
-      <c r="H53" s="6">
+      <c r="H53" s="7">
         <v>1.4</v>
       </c>
-      <c r="I53" s="6" t="s">
+      <c r="I53" s="7" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A54" s="7"/>
+      <c r="A54" s="6"/>
       <c r="B54" s="3"/>
-      <c r="C54" s="6"/>
-      <c r="D54" s="6"/>
-      <c r="E54" s="6"/>
-      <c r="F54" s="6"/>
-      <c r="G54" s="6"/>
-      <c r="H54" s="6"/>
-      <c r="I54" s="6"/>
+      <c r="C54" s="7"/>
+      <c r="D54" s="7"/>
+      <c r="E54" s="7"/>
+      <c r="F54" s="7"/>
+      <c r="G54" s="7"/>
+      <c r="H54" s="7"/>
+      <c r="I54" s="7"/>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A55" s="7"/>
+      <c r="A55" s="6"/>
       <c r="B55" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C55" s="6"/>
-      <c r="D55" s="6"/>
-      <c r="E55" s="6"/>
-      <c r="F55" s="6"/>
-      <c r="G55" s="6"/>
-      <c r="H55" s="6"/>
-      <c r="I55" s="6"/>
+      <c r="C55" s="7"/>
+      <c r="D55" s="7"/>
+      <c r="E55" s="7"/>
+      <c r="F55" s="7"/>
+      <c r="G55" s="7"/>
+      <c r="H55" s="7"/>
+      <c r="I55" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="137">
-    <mergeCell ref="A5:A7"/>
-    <mergeCell ref="C5:C7"/>
-    <mergeCell ref="D5:D7"/>
-    <mergeCell ref="E5:E7"/>
-    <mergeCell ref="F5:F7"/>
-    <mergeCell ref="G5:G7"/>
-    <mergeCell ref="H5:H7"/>
-    <mergeCell ref="I5:I7"/>
-    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="H50:H52"/>
+    <mergeCell ref="I50:I52"/>
+    <mergeCell ref="A53:A55"/>
+    <mergeCell ref="C53:C55"/>
+    <mergeCell ref="D53:D55"/>
+    <mergeCell ref="E53:E55"/>
+    <mergeCell ref="F53:F55"/>
+    <mergeCell ref="G53:G55"/>
+    <mergeCell ref="H53:H55"/>
+    <mergeCell ref="I53:I55"/>
+    <mergeCell ref="A50:A52"/>
+    <mergeCell ref="C50:C52"/>
+    <mergeCell ref="D50:D52"/>
+    <mergeCell ref="E50:E52"/>
+    <mergeCell ref="F50:F52"/>
+    <mergeCell ref="G50:G52"/>
+    <mergeCell ref="H44:H46"/>
+    <mergeCell ref="I44:I46"/>
+    <mergeCell ref="A47:A49"/>
+    <mergeCell ref="C47:C49"/>
+    <mergeCell ref="D47:D49"/>
+    <mergeCell ref="E47:E49"/>
+    <mergeCell ref="F47:F49"/>
+    <mergeCell ref="G47:G49"/>
+    <mergeCell ref="H47:H49"/>
+    <mergeCell ref="I47:I49"/>
+    <mergeCell ref="A44:A46"/>
+    <mergeCell ref="C44:C46"/>
+    <mergeCell ref="D44:D46"/>
+    <mergeCell ref="E44:E46"/>
+    <mergeCell ref="F44:F46"/>
+    <mergeCell ref="G44:G46"/>
+    <mergeCell ref="H38:H40"/>
+    <mergeCell ref="I38:I40"/>
+    <mergeCell ref="A41:A43"/>
+    <mergeCell ref="C41:C43"/>
+    <mergeCell ref="D41:D43"/>
+    <mergeCell ref="E41:E43"/>
+    <mergeCell ref="F41:F43"/>
+    <mergeCell ref="G41:G43"/>
+    <mergeCell ref="H41:H43"/>
+    <mergeCell ref="I41:I43"/>
+    <mergeCell ref="A38:A40"/>
+    <mergeCell ref="C38:C40"/>
+    <mergeCell ref="D38:D40"/>
+    <mergeCell ref="E38:E40"/>
+    <mergeCell ref="F38:F40"/>
+    <mergeCell ref="G38:G40"/>
+    <mergeCell ref="H32:H34"/>
+    <mergeCell ref="I32:I34"/>
+    <mergeCell ref="A35:A37"/>
+    <mergeCell ref="C35:C37"/>
+    <mergeCell ref="D35:D37"/>
+    <mergeCell ref="E35:E37"/>
+    <mergeCell ref="F35:F37"/>
+    <mergeCell ref="G35:G37"/>
+    <mergeCell ref="H35:H37"/>
+    <mergeCell ref="I35:I37"/>
+    <mergeCell ref="A32:A34"/>
+    <mergeCell ref="C32:C34"/>
+    <mergeCell ref="D32:D34"/>
+    <mergeCell ref="E32:E34"/>
+    <mergeCell ref="F32:F34"/>
+    <mergeCell ref="G32:G34"/>
+    <mergeCell ref="H26:H28"/>
+    <mergeCell ref="I26:I28"/>
+    <mergeCell ref="A29:A31"/>
+    <mergeCell ref="C29:C31"/>
+    <mergeCell ref="D29:D31"/>
+    <mergeCell ref="E29:E31"/>
+    <mergeCell ref="F29:F31"/>
+    <mergeCell ref="G29:G31"/>
+    <mergeCell ref="H29:H31"/>
+    <mergeCell ref="I29:I31"/>
+    <mergeCell ref="A26:A28"/>
+    <mergeCell ref="C26:C28"/>
+    <mergeCell ref="D26:D28"/>
+    <mergeCell ref="E26:E28"/>
+    <mergeCell ref="F26:F28"/>
+    <mergeCell ref="G26:G28"/>
+    <mergeCell ref="H20:H22"/>
+    <mergeCell ref="I20:I22"/>
+    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="C23:C25"/>
+    <mergeCell ref="D23:D25"/>
+    <mergeCell ref="E23:E25"/>
+    <mergeCell ref="F23:F25"/>
+    <mergeCell ref="G23:G25"/>
+    <mergeCell ref="H23:H25"/>
+    <mergeCell ref="I23:I25"/>
+    <mergeCell ref="A20:A22"/>
+    <mergeCell ref="C20:C22"/>
+    <mergeCell ref="D20:D22"/>
+    <mergeCell ref="E20:E22"/>
+    <mergeCell ref="F20:F22"/>
+    <mergeCell ref="G20:G22"/>
+    <mergeCell ref="H14:H16"/>
+    <mergeCell ref="I14:I16"/>
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="C17:C19"/>
+    <mergeCell ref="D17:D19"/>
+    <mergeCell ref="E17:E19"/>
+    <mergeCell ref="F17:F19"/>
+    <mergeCell ref="G17:G19"/>
+    <mergeCell ref="H17:H19"/>
+    <mergeCell ref="I17:I19"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="D14:D16"/>
+    <mergeCell ref="E14:E16"/>
+    <mergeCell ref="F14:F16"/>
+    <mergeCell ref="G14:G16"/>
     <mergeCell ref="H8:H10"/>
     <mergeCell ref="I8:I10"/>
     <mergeCell ref="A11:A13"/>
@@ -1706,118 +1809,15 @@
     <mergeCell ref="E8:E10"/>
     <mergeCell ref="F8:F10"/>
     <mergeCell ref="G8:G10"/>
-    <mergeCell ref="H14:H16"/>
-    <mergeCell ref="I14:I16"/>
-    <mergeCell ref="A17:A19"/>
-    <mergeCell ref="C17:C19"/>
-    <mergeCell ref="D17:D19"/>
-    <mergeCell ref="E17:E19"/>
-    <mergeCell ref="F17:F19"/>
-    <mergeCell ref="G17:G19"/>
-    <mergeCell ref="H17:H19"/>
-    <mergeCell ref="I17:I19"/>
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="C14:C16"/>
-    <mergeCell ref="D14:D16"/>
-    <mergeCell ref="E14:E16"/>
-    <mergeCell ref="F14:F16"/>
-    <mergeCell ref="G14:G16"/>
-    <mergeCell ref="H20:H22"/>
-    <mergeCell ref="I20:I22"/>
-    <mergeCell ref="A23:A25"/>
-    <mergeCell ref="C23:C25"/>
-    <mergeCell ref="D23:D25"/>
-    <mergeCell ref="E23:E25"/>
-    <mergeCell ref="F23:F25"/>
-    <mergeCell ref="G23:G25"/>
-    <mergeCell ref="H23:H25"/>
-    <mergeCell ref="I23:I25"/>
-    <mergeCell ref="A20:A22"/>
-    <mergeCell ref="C20:C22"/>
-    <mergeCell ref="D20:D22"/>
-    <mergeCell ref="E20:E22"/>
-    <mergeCell ref="F20:F22"/>
-    <mergeCell ref="G20:G22"/>
-    <mergeCell ref="H26:H28"/>
-    <mergeCell ref="I26:I28"/>
-    <mergeCell ref="A29:A31"/>
-    <mergeCell ref="C29:C31"/>
-    <mergeCell ref="D29:D31"/>
-    <mergeCell ref="E29:E31"/>
-    <mergeCell ref="F29:F31"/>
-    <mergeCell ref="G29:G31"/>
-    <mergeCell ref="H29:H31"/>
-    <mergeCell ref="I29:I31"/>
-    <mergeCell ref="A26:A28"/>
-    <mergeCell ref="C26:C28"/>
-    <mergeCell ref="D26:D28"/>
-    <mergeCell ref="E26:E28"/>
-    <mergeCell ref="F26:F28"/>
-    <mergeCell ref="G26:G28"/>
-    <mergeCell ref="H32:H34"/>
-    <mergeCell ref="I32:I34"/>
-    <mergeCell ref="A35:A37"/>
-    <mergeCell ref="C35:C37"/>
-    <mergeCell ref="D35:D37"/>
-    <mergeCell ref="E35:E37"/>
-    <mergeCell ref="F35:F37"/>
-    <mergeCell ref="G35:G37"/>
-    <mergeCell ref="H35:H37"/>
-    <mergeCell ref="I35:I37"/>
-    <mergeCell ref="A32:A34"/>
-    <mergeCell ref="C32:C34"/>
-    <mergeCell ref="D32:D34"/>
-    <mergeCell ref="E32:E34"/>
-    <mergeCell ref="F32:F34"/>
-    <mergeCell ref="G32:G34"/>
-    <mergeCell ref="H38:H40"/>
-    <mergeCell ref="I38:I40"/>
-    <mergeCell ref="A41:A43"/>
-    <mergeCell ref="C41:C43"/>
-    <mergeCell ref="D41:D43"/>
-    <mergeCell ref="E41:E43"/>
-    <mergeCell ref="F41:F43"/>
-    <mergeCell ref="G41:G43"/>
-    <mergeCell ref="H41:H43"/>
-    <mergeCell ref="I41:I43"/>
-    <mergeCell ref="A38:A40"/>
-    <mergeCell ref="C38:C40"/>
-    <mergeCell ref="D38:D40"/>
-    <mergeCell ref="E38:E40"/>
-    <mergeCell ref="F38:F40"/>
-    <mergeCell ref="G38:G40"/>
-    <mergeCell ref="H44:H46"/>
-    <mergeCell ref="I44:I46"/>
-    <mergeCell ref="A47:A49"/>
-    <mergeCell ref="C47:C49"/>
-    <mergeCell ref="D47:D49"/>
-    <mergeCell ref="E47:E49"/>
-    <mergeCell ref="F47:F49"/>
-    <mergeCell ref="G47:G49"/>
-    <mergeCell ref="H47:H49"/>
-    <mergeCell ref="I47:I49"/>
-    <mergeCell ref="A44:A46"/>
-    <mergeCell ref="C44:C46"/>
-    <mergeCell ref="D44:D46"/>
-    <mergeCell ref="E44:E46"/>
-    <mergeCell ref="F44:F46"/>
-    <mergeCell ref="G44:G46"/>
-    <mergeCell ref="H50:H52"/>
-    <mergeCell ref="I50:I52"/>
-    <mergeCell ref="A53:A55"/>
-    <mergeCell ref="C53:C55"/>
-    <mergeCell ref="D53:D55"/>
-    <mergeCell ref="E53:E55"/>
-    <mergeCell ref="F53:F55"/>
-    <mergeCell ref="G53:G55"/>
-    <mergeCell ref="H53:H55"/>
-    <mergeCell ref="I53:I55"/>
-    <mergeCell ref="A50:A52"/>
-    <mergeCell ref="C50:C52"/>
-    <mergeCell ref="D50:D52"/>
-    <mergeCell ref="E50:E52"/>
-    <mergeCell ref="F50:F52"/>
-    <mergeCell ref="G50:G52"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="D5:D7"/>
+    <mergeCell ref="E5:E7"/>
+    <mergeCell ref="F5:F7"/>
+    <mergeCell ref="G5:G7"/>
+    <mergeCell ref="H5:H7"/>
+    <mergeCell ref="I5:I7"/>
+    <mergeCell ref="A2:A4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
adding new archer enemy
</commit_message>
<xml_diff>
--- a/initial_enemies_stats.xlsx
+++ b/initial_enemies_stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\godot\rpg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AC9767A-F8CE-4DB6-B255-19EC89A3D597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{694259AD-7CDF-4BEB-AE26-B3E7DBBE9FEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,16 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="62">
-  <si>
-    <t>Skeleton Warrior</t>
-  </si>
-  <si>
-    <t>Ironclad Guard</t>
-  </si>
-  <si>
-    <t>Walkin' Shark</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="64">
   <si>
     <t>Round Puffer</t>
   </si>
@@ -42,39 +33,15 @@
     <t>Bone Witch Doctor</t>
   </si>
   <si>
-    <t>Goblin Lancer</t>
-  </si>
-  <si>
-    <t>Goblin Torchbearer</t>
-  </si>
-  <si>
     <t>Wild Ratfolk</t>
   </si>
   <si>
-    <t>Shadow Weaver</t>
-  </si>
-  <si>
-    <t>Emerald Drake</t>
-  </si>
-  <si>
     <t>Acorn Gnome</t>
   </si>
   <si>
     <t>Panda Monk</t>
   </si>
   <si>
-    <t>Ancient Snapping Turtle</t>
-  </si>
-  <si>
-    <t>Grizzly Maul</t>
-  </si>
-  <si>
-    <t>Viper</t>
-  </si>
-  <si>
-    <t>Hooded Rogue</t>
-  </si>
-  <si>
     <t>Ligne (Image)</t>
   </si>
   <si>
@@ -171,18 +138,9 @@
     <t>1.3s</t>
   </si>
   <si>
-    <t>180 (Ranged)</t>
-  </si>
-  <si>
-    <t>Minotaur Executioner (Mini-Boss)</t>
-  </si>
-  <si>
     <t>9.5 (Poison)</t>
   </si>
   <si>
-    <t>120 (Ranged)</t>
-  </si>
-  <si>
     <t>140 (Ranged)</t>
   </si>
   <si>
@@ -211,6 +169,54 @@
   </si>
   <si>
     <t>50.0 (5.0x Boss)</t>
+  </si>
+  <si>
+    <t>Bone Scrappy</t>
+  </si>
+  <si>
+    <t>Goblin Spearhead</t>
+  </si>
+  <si>
+    <t>Pot-helm Brawler</t>
+  </si>
+  <si>
+    <t>Landfin</t>
+  </si>
+  <si>
+    <t>320 (Ranged)</t>
+  </si>
+  <si>
+    <t>Goblin Pyromancer</t>
+  </si>
+  <si>
+    <t>Minotaur Executioner (Capitain)</t>
+  </si>
+  <si>
+    <t>Dungeon Spider</t>
+  </si>
+  <si>
+    <t>Serpent Sage</t>
+  </si>
+  <si>
+    <t>Iron-Shell Tortoise</t>
+  </si>
+  <si>
+    <t>Dire Bear</t>
+  </si>
+  <si>
+    <t>Sand Snake</t>
+  </si>
+  <si>
+    <t>Shadow Bandit</t>
+  </si>
+  <si>
+    <t>300 (Ranged)</t>
+  </si>
+  <si>
+    <t>230 (Ranged)</t>
+  </si>
+  <si>
+    <t>190 (Ranged)</t>
   </si>
 </sst>
 </file>
@@ -611,45 +617,45 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="C2" s="1">
         <v>100</v>
       </c>
       <c r="D2" s="1">
-        <v>28</v>
+        <v>65</v>
       </c>
       <c r="E2" s="1">
         <v>65</v>
@@ -661,10 +667,10 @@
         <v>1.2</v>
       </c>
       <c r="H2" s="1">
-        <v>0.8</v>
+        <v>0.36699999999999999</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -681,7 +687,7 @@
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -693,16 +699,16 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="C5" s="1">
         <v>160</v>
       </c>
       <c r="D5" s="1">
-        <v>32</v>
+        <v>75</v>
       </c>
       <c r="E5" s="1">
         <v>45</v>
@@ -714,10 +720,10 @@
         <v>1.5</v>
       </c>
       <c r="H5" s="1">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -734,7 +740,7 @@
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="1" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -746,16 +752,16 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>2</v>
+        <v>51</v>
       </c>
       <c r="C8" s="1">
         <v>110</v>
       </c>
-      <c r="D8" s="1">
-        <v>35</v>
+      <c r="D8" s="1" t="s">
+        <v>52</v>
       </c>
       <c r="E8" s="1">
         <v>75</v>
@@ -767,10 +773,10 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="H8" s="1">
-        <v>0.75</v>
+        <v>0.26700000000000002</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
@@ -787,7 +793,7 @@
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="1" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -799,16 +805,16 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C11" s="1">
         <v>80</v>
       </c>
-      <c r="D11" s="1">
-        <v>24</v>
+      <c r="D11" s="1" t="s">
+        <v>61</v>
       </c>
       <c r="E11" s="1">
         <v>40</v>
@@ -823,7 +829,7 @@
         <v>0.6</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
@@ -840,7 +846,7 @@
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="1" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
@@ -852,16 +858,16 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C14" s="1">
         <v>75</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="E14" s="1">
         <v>50</v>
@@ -873,10 +879,10 @@
         <v>1.4</v>
       </c>
       <c r="H14" s="1">
-        <v>0.9</v>
+        <v>0.33300000000000002</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
@@ -893,7 +899,7 @@
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="1" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
@@ -905,16 +911,16 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="C17" s="1">
         <v>90</v>
       </c>
       <c r="D17" s="1">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="E17" s="1">
         <v>70</v>
@@ -923,13 +929,13 @@
         <v>9</v>
       </c>
       <c r="G17" s="1">
-        <v>1</v>
+        <v>1.8</v>
       </c>
       <c r="H17" s="1">
-        <v>0.7</v>
+        <v>0.23300000000000001</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
@@ -946,7 +952,7 @@
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="1" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
@@ -958,16 +964,16 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>6</v>
+        <v>53</v>
       </c>
       <c r="C20" s="1">
         <v>85</v>
       </c>
       <c r="D20" s="1">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="E20" s="1">
         <v>80</v>
@@ -979,10 +985,10 @@
         <v>0.9</v>
       </c>
       <c r="H20" s="1">
-        <v>0.65</v>
+        <v>0.23330000000000001</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
@@ -999,7 +1005,7 @@
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="1" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
@@ -1011,16 +1017,16 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C23" s="1">
         <v>450</v>
       </c>
       <c r="D23" s="1">
-        <v>48</v>
+        <v>85</v>
       </c>
       <c r="E23" s="1">
         <v>40</v>
@@ -1029,13 +1035,13 @@
         <v>25</v>
       </c>
       <c r="G23" s="1">
-        <v>2</v>
+        <v>2.8</v>
       </c>
       <c r="H23" s="1">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
@@ -1052,7 +1058,7 @@
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="1" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
@@ -1064,16 +1070,16 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C26" s="1">
         <v>65</v>
       </c>
-      <c r="D26" s="1">
-        <v>22</v>
+      <c r="D26" s="1" t="s">
+        <v>38</v>
       </c>
       <c r="E26" s="1">
         <v>90</v>
@@ -1088,7 +1094,7 @@
         <v>0.5</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
@@ -1105,7 +1111,7 @@
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="1" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
@@ -1117,31 +1123,31 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>8</v>
+        <v>55</v>
       </c>
       <c r="C29" s="1">
         <v>95</v>
       </c>
       <c r="D29" s="1">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="E29" s="1">
         <v>70</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="G29" s="1">
         <v>1.1000000000000001</v>
       </c>
       <c r="H29" s="1">
-        <v>0.7</v>
+        <v>0.26700000000000002</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
@@ -1158,7 +1164,7 @@
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="1" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
@@ -1170,16 +1176,16 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>9</v>
+        <v>56</v>
       </c>
       <c r="C32" s="1">
         <v>130</v>
       </c>
-      <c r="D32" s="1" t="s">
-        <v>51</v>
+      <c r="D32" s="1">
+        <v>55</v>
       </c>
       <c r="E32" s="1">
         <v>55</v>
@@ -1191,10 +1197,10 @@
         <v>1.3</v>
       </c>
       <c r="H32" s="1">
-        <v>0.85</v>
+        <v>0.3</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
@@ -1211,7 +1217,7 @@
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="1" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
@@ -1223,16 +1229,16 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="C35" s="1">
         <v>60</v>
       </c>
-      <c r="D35" s="1" t="s">
-        <v>52</v>
+      <c r="D35" s="1">
+        <v>65</v>
       </c>
       <c r="E35" s="1">
         <v>85</v>
@@ -1244,10 +1250,10 @@
         <v>0.8</v>
       </c>
       <c r="H35" s="1">
-        <v>0.55000000000000004</v>
+        <v>0.23300000000000001</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
@@ -1264,7 +1270,7 @@
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="1" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
@@ -1276,31 +1282,31 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C38" s="1">
         <v>140</v>
       </c>
       <c r="D38" s="1">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="E38" s="1">
         <v>60</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="G38" s="1">
-        <v>0.9</v>
+        <v>2.5</v>
       </c>
       <c r="H38" s="1">
-        <v>0.8</v>
+        <v>0.43330000000000002</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
@@ -1317,7 +1323,7 @@
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
       <c r="B40" s="1" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
@@ -1329,16 +1335,16 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="C41" s="1">
         <v>220</v>
       </c>
       <c r="D41" s="1">
-        <v>26</v>
+        <v>120</v>
       </c>
       <c r="E41" s="1">
         <v>30</v>
@@ -1350,10 +1356,10 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="H41" s="1">
-        <v>1.1000000000000001</v>
+        <v>0.33300000000000002</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.3">
@@ -1370,7 +1376,7 @@
     <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="1" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="C43" s="1"/>
       <c r="D43" s="1"/>
@@ -1382,16 +1388,16 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>13</v>
+        <v>58</v>
       </c>
       <c r="C44" s="1">
         <v>180</v>
       </c>
       <c r="D44" s="1">
-        <v>36</v>
+        <v>77</v>
       </c>
       <c r="E44" s="1">
         <v>50</v>
@@ -1403,10 +1409,10 @@
         <v>1.6</v>
       </c>
       <c r="H44" s="1">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.3">
@@ -1423,7 +1429,7 @@
     <row r="46" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
       <c r="B46" s="1" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="C46" s="1"/>
       <c r="D46" s="1"/>
@@ -1435,16 +1441,16 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>14</v>
+        <v>59</v>
       </c>
       <c r="C47" s="1">
         <v>70</v>
       </c>
       <c r="D47" s="1">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="E47" s="1">
         <v>80</v>
@@ -1459,7 +1465,7 @@
         <v>0.6</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.3">
@@ -1476,7 +1482,7 @@
     <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
       <c r="B49" s="1" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="C49" s="1"/>
       <c r="D49" s="1"/>
@@ -1488,16 +1494,16 @@
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="C50" s="1">
         <v>85</v>
       </c>
       <c r="D50" s="1">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="E50" s="1">
         <v>95</v>
@@ -1509,10 +1515,10 @@
         <v>0.75</v>
       </c>
       <c r="H50" s="1">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="I50" s="1" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.3">
@@ -1529,7 +1535,7 @@
     <row r="52" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A52" s="1"/>
       <c r="B52" s="1" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="C52" s="1"/>
       <c r="D52" s="1"/>
@@ -1541,16 +1547,16 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="C53" s="1">
         <v>150</v>
       </c>
-      <c r="D53" s="1">
-        <v>20</v>
+      <c r="D53" s="1" t="s">
+        <v>63</v>
       </c>
       <c r="E53" s="1">
         <v>25</v>
@@ -1565,7 +1571,7 @@
         <v>0.8</v>
       </c>
       <c r="I53" s="1" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.3">
@@ -1582,7 +1588,7 @@
     <row r="55" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
       <c r="B55" s="1" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="C55" s="1"/>
       <c r="D55" s="1"/>
@@ -1594,31 +1600,31 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="C56" s="1">
         <v>55</v>
       </c>
       <c r="D56" s="1">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E56" s="1">
         <v>110</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="G56" s="1">
         <v>0.6</v>
       </c>
       <c r="H56" s="1">
-        <v>0.45</v>
+        <v>0.23300000000000001</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.3">
@@ -1635,7 +1641,7 @@
     <row r="58" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A58" s="1"/>
       <c r="B58" s="1" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="C58" s="1"/>
       <c r="D58" s="1"/>
@@ -1647,10 +1653,10 @@
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="C59" s="1">
         <v>50</v>
@@ -1668,10 +1674,10 @@
         <v>0.5</v>
       </c>
       <c r="H59" s="1">
-        <v>0.4</v>
+        <v>0.36699999999999999</v>
       </c>
       <c r="I59" s="1" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.3">
@@ -1688,7 +1694,7 @@
     <row r="61" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A61" s="1"/>
       <c r="B61" s="1" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="C61" s="1"/>
       <c r="D61" s="1"/>
@@ -1700,10 +1706,10 @@
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C62" s="1">
         <v>120</v>
@@ -1718,13 +1724,13 @@
         <v>12.5</v>
       </c>
       <c r="G62" s="1">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="H62" s="1">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="I62" s="1" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.3">
@@ -1741,7 +1747,7 @@
     <row r="64" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A64" s="1"/>
       <c r="B64" s="1" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="C64" s="1"/>
       <c r="D64" s="1"/>
@@ -1753,10 +1759,10 @@
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="C65" s="1">
         <v>800</v>
@@ -1768,7 +1774,7 @@
         <v>35</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="G65" s="1">
         <v>2.5</v>
@@ -1777,7 +1783,7 @@
         <v>1.4</v>
       </c>
       <c r="I65" s="1" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.3">
@@ -1794,7 +1800,7 @@
     <row r="67" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A67" s="1"/>
       <c r="B67" s="1" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="C67" s="1"/>
       <c r="D67" s="1"/>

</xml_diff>